<commit_message>
Update excel untittests for rate helpers.
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_ratehelpers.xlsx
+++ b/tests/workbooks/test_ratehelpers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA258476-C7E2-42A2-883C-AB21421C035D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5F18A0-4DE7-4C93-816A-69FC7F3E51BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{60DEDABF-8191-4F74-809B-551F46E87618}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{60DEDABF-8191-4F74-809B-551F46E87618}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview Tabs" sheetId="18" r:id="rId1"/>
@@ -614,7 +614,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -657,6 +660,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -681,10 +691,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -715,8 +726,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1150,9 +1168,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1160,10 +1178,10 @@
         <v>33</v>
       </c>
       <c r="B4" s="12">
-        <v>0.6</v>
+        <v>95.5</v>
       </c>
       <c r="C4" s="12">
-        <v>0.1</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1192,13 +1210,13 @@
       <c r="A7" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="12" t="str">
-        <f>_xll.qlOvernightIndex("MyIndex",3,"EUR","TARGET","actual360")</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIindexFutureRateHelper!R7C2OvernightIndex,A</v>
-      </c>
-      <c r="C7" s="12" t="str">
-        <f>_xll.qlOvernightIndex("MyIndex",3,"EUR","TARGET","actual360")</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIindexFutureRateHelper!R7C3OvernightIndex,A</v>
+      <c r="B7" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIndex("MyIndex",3,"EUR","TARGET","actual360")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIndex("MyIndex",3,"EUR","TARGET","actual360")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1224,104 +1242,104 @@
       <c r="A10" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="12" t="str">
-        <f>_xll.qlOvernightIndexFutureRateHelper(B4,B5,B6,B7,B8)</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIindexFutureRateHelper!R10C2OvernightIndexFutureRateHelper,A</v>
-      </c>
-      <c r="C10" s="12" t="str">
-        <f>_xll.qlOvernightIndexFutureRateHelper(C4,C5,C6,C7,C8,C9)</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIindexFutureRateHelper!R10C3OvernightIndexFutureRateHelper,A</v>
+      <c r="B10" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIndexFutureRateHelper(B4,B5,B6,B7,B8)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C10" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIndexFutureRateHelper(C4,C5,C6,C7,C8,C9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="12">
-        <f>_xll.qlRateHelperQuote(B10)</f>
-        <v>0.6</v>
-      </c>
-      <c r="C11" s="12">
-        <f>_xll.qlRateHelperQuote(C10)</f>
-        <v>0.1</v>
+      <c r="B11" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C11" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="11">
-        <f>_xll.qlRateHelperLatestDate(B10)</f>
-        <v>45755</v>
-      </c>
-      <c r="C12" s="11">
-        <f>_xll.qlRateHelperLatestDate(C10)</f>
-        <v>45755</v>
+      <c r="B12" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C12" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B10)</f>
-        <v>45663</v>
-      </c>
-      <c r="C13" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C10)</f>
-        <v>45663</v>
+      <c r="B13" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C13" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B10)</f>
-        <v>45755</v>
-      </c>
-      <c r="C14" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C10)</f>
-        <v>45755</v>
+      <c r="B14" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C14" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B10)</f>
-        <v>45755</v>
-      </c>
-      <c r="C15" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C10)</f>
-        <v>45755</v>
+      <c r="B15" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C15" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="11">
-        <f>_xll.qlRateHelperPillarDate(B10)</f>
-        <v>45755</v>
-      </c>
-      <c r="C16" s="11">
-        <f>_xll.qlRateHelperPillarDate(C10)</f>
-        <v>45755</v>
+      <c r="B16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="12">
-        <f>_xll.qlOvernightIndexFutureRateHelperConvexityAdjustment(B10)</f>
-        <v>0.5</v>
-      </c>
-      <c r="C17" s="12">
-        <f>_xll.qlOvernightIndexFutureRateHelperConvexityAdjustment(C10)</f>
-        <v>0.9</v>
+      <c r="B17" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIndexFutureRateHelperConvexityAdjustment(B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C17" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIndexFutureRateHelperConvexityAdjustment(C10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -1350,9 +1368,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1360,7 +1378,7 @@
         <v>33</v>
       </c>
       <c r="B4" s="12">
-        <v>0.2</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1396,63 +1414,63 @@
       <c r="A9" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="12" t="str">
-        <f>_xll.qlSofrFutureRateHelper(B4,B5,B6,B7)</f>
-        <v>欣[test_ratehelpers.xlsx]SofrFutureRateHelper!R9C2SofrFutureRateHelper,A</v>
+      <c r="B9" s="12" t="e">
+        <f ca="1">_xll.qlSofrFutureRateHelper(B4,B5,B6,B7)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="12">
-        <f>_xll.qlRateHelperQuote(B9)</f>
-        <v>0.2</v>
+      <c r="B10" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="11">
-        <f>_xll.qlRateHelperLatestDate(B9)</f>
-        <v>45778</v>
+      <c r="B11" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B9)</f>
-        <v>45748</v>
+      <c r="B12" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B9)</f>
-        <v>45778</v>
+      <c r="B13" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B9)</f>
-        <v>45778</v>
+      <c r="B14" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="11">
-        <f>_xll.qlRateHelperPillarDate(B9)</f>
-        <v>45778</v>
+      <c r="B15" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B9)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -1483,20 +1501,20 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="12">
-        <v>0.4</v>
-      </c>
-      <c r="C4" s="12">
-        <v>0.4</v>
+      <c r="B4" s="18">
+        <v>0.04</v>
+      </c>
+      <c r="C4" s="18">
+        <v>0.04</v>
       </c>
       <c r="D4" s="12"/>
     </row>
@@ -1528,13 +1546,13 @@
       <c r="A7" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="D7" s="12"/>
     </row>
@@ -1590,13 +1608,13 @@
       <c r="A12" t="s">
         <v>164</v>
       </c>
-      <c r="B12" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencySwapR!R12C2Euribor,A</v>
-      </c>
-      <c r="C12" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencySwapR!R12C3Euribor,A</v>
+      <c r="B12" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C12" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="D12" s="12"/>
     </row>
@@ -1604,13 +1622,13 @@
       <c r="A13" t="s">
         <v>162</v>
       </c>
-      <c r="B13" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencySwapR!R13C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C13" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencySwapR!R13C3YieldTermStructureHandle,A</v>
+      <c r="B13" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C13" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="D13" s="12"/>
     </row>
@@ -1639,91 +1657,91 @@
       <c r="A16" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="12" t="str">
-        <f>_xll.qlConstNotionalCrossCurrencySwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13,B14)</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencySwapR!R16C2ConstNotionalCrossCurrencySwapRateHelper,A</v>
-      </c>
-      <c r="C16" s="12" t="str">
-        <f>_xll.qlConstNotionalCrossCurrencySwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15)</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencySwapR!R16C3ConstNotionalCrossCurrencySwapRateHelper,A</v>
+      <c r="B16" s="12" t="e">
+        <f ca="1">_xll.qlConstNotionalCrossCurrencySwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13,B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C16" s="12" t="e">
+        <f ca="1">_xll.qlConstNotionalCrossCurrencySwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="12">
-        <f>_xll.qlRateHelperQuote(B16)</f>
-        <v>0.4</v>
-      </c>
-      <c r="C17" s="12">
-        <f>_xll.qlRateHelperQuote(C16)</f>
-        <v>0.4</v>
+      <c r="B17" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B16)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C17" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C16)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="11">
-        <f>_xll.qlRateHelperLatestDate(B16)</f>
-        <v>45846</v>
-      </c>
-      <c r="C18" s="11">
-        <f>_xll.qlRateHelperLatestDate(C16)</f>
-        <v>45847</v>
+      <c r="B18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B16)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C16)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B16)</f>
-        <v>45665</v>
-      </c>
-      <c r="C19" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C16)</f>
-        <v>45665</v>
+      <c r="B19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B16)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C16)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B16)</f>
-        <v>45846</v>
-      </c>
-      <c r="C20" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C16)</f>
-        <v>45846</v>
+      <c r="B20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B16)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C16)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B16)</f>
-        <v>45846</v>
-      </c>
-      <c r="C21" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C16)</f>
-        <v>45847</v>
+      <c r="B21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B16)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C16)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="11">
-        <f>_xll.qlRateHelperPillarDate(B16)</f>
-        <v>45846</v>
-      </c>
-      <c r="C22" s="11">
-        <f>_xll.qlRateHelperPillarDate(C16)</f>
-        <v>45847</v>
+      <c r="B22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B16)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C16)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -1754,9 +1772,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1764,10 +1782,10 @@
         <v>93</v>
       </c>
       <c r="B4" s="12">
-        <v>0.5</v>
+        <v>1E-3</v>
       </c>
       <c r="C4" s="12">
-        <v>0.5</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1796,13 +1814,13 @@
       <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1831,39 +1849,39 @@
       <c r="A10" t="s">
         <v>165</v>
       </c>
-      <c r="B10" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R10C2Euribor,A</v>
-      </c>
-      <c r="C10" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R10C3Euribor,A</v>
+      <c r="B10" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C10" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>166</v>
       </c>
-      <c r="B11" s="12" t="str">
-        <f>_xll.qlEuribor("6M")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R11C2Euribor,A</v>
-      </c>
-      <c r="C11" s="12" t="str">
-        <f>_xll.qlEuribor("6M")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R11C3Euribor,A</v>
+      <c r="B11" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("6M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C11" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("6M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>162</v>
       </c>
-      <c r="B12" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R12C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C12" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R12C3YieldTermStructureHandle,A</v>
+      <c r="B12" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C12" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1911,91 +1929,91 @@
       <c r="A17" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="12" t="str">
-        <f>_xll.qlConstNotionalCrossCurrencyBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15)</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R17C2ConstNotionalCrossCurrencyBasisSwapRateHelper,A</v>
-      </c>
-      <c r="C17" s="12" t="str">
-        <f>_xll.qlConstNotionalCrossCurrencyBasisSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,C16)</f>
-        <v>欣[test_ratehelpers.xlsx]ConstNotionalCrossCurrencyBasis!R17C3ConstNotionalCrossCurrencyBasisSwapRateHelper,A</v>
+      <c r="B17" s="12" t="e">
+        <f ca="1">_xll.qlConstNotionalCrossCurrencyBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C17" s="12" t="e">
+        <f ca="1">_xll.qlConstNotionalCrossCurrencyBasisSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,C16)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="12">
-        <f>_xll.qlRateHelperQuote(B17)</f>
-        <v>0.5</v>
-      </c>
-      <c r="C18" s="12">
-        <f>_xll.qlRateHelperQuote(C17)</f>
-        <v>0.5</v>
+      <c r="B18" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B17)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C18" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C17)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="11">
-        <f>_xll.qlRateHelperLatestDate(B17)</f>
-        <v>45754</v>
-      </c>
-      <c r="C19" s="11">
-        <f>_xll.qlRateHelperLatestDate(C17)</f>
-        <v>45755</v>
+      <c r="B19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B17)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C17)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B17)</f>
-        <v>45663</v>
-      </c>
-      <c r="C20" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C17)</f>
-        <v>45663</v>
+      <c r="B20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B17)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C17)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B17)</f>
-        <v>45754</v>
-      </c>
-      <c r="C21" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C17)</f>
-        <v>45754</v>
+      <c r="B21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B17)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C17)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B17)</f>
-        <v>45754</v>
-      </c>
-      <c r="C22" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C17)</f>
-        <v>45755</v>
+      <c r="B22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B17)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C17)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="11">
-        <f>_xll.qlRateHelperPillarDate(B17)</f>
-        <v>45754</v>
-      </c>
-      <c r="C23" s="11">
-        <f>_xll.qlRateHelperPillarDate(C17)</f>
-        <v>45755</v>
+      <c r="B23" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B17)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C23" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C17)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -2026,9 +2044,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2036,10 +2054,10 @@
         <v>93</v>
       </c>
       <c r="B4" s="12">
-        <v>0.8</v>
+        <v>1E-3</v>
       </c>
       <c r="C4" s="12">
-        <v>0.8</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2068,13 +2086,13 @@
       <c r="A7" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2103,39 +2121,39 @@
       <c r="A10" t="s">
         <v>167</v>
       </c>
-      <c r="B10" s="12" t="str">
-        <f>_xll.qlCADLibor("6m")</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R10C2CADLibor,A</v>
-      </c>
-      <c r="C10" s="12" t="str">
-        <f>_xll.qlCADLibor("6m")</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R10C3CADLibor,A</v>
+      <c r="B10" s="12" t="e">
+        <f ca="1">_xll.qlCADLibor("6m")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C10" s="12" t="e">
+        <f ca="1">_xll.qlCADLibor("6m")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>166</v>
       </c>
-      <c r="B11" s="12" t="str">
-        <f>_xll.qlEuribor("6M")</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R11C2Euribor,A</v>
-      </c>
-      <c r="C11" s="12" t="str">
-        <f>_xll.qlEuribor("6M")</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R11C3Euribor,A</v>
+      <c r="B11" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("6M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C11" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("6M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>162</v>
       </c>
-      <c r="B12" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R12C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C12" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R12C3YieldTermStructureHandle,A</v>
+      <c r="B12" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C12" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2194,91 +2212,91 @@
       <c r="A18" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="12" t="str">
-        <f>_xll.qlMtMCrossCurrencyBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16)</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R18C2MtMCrossCurrencyBasisSwapRateHelper,A</v>
-      </c>
-      <c r="C18" s="12" t="str">
-        <f>_xll.qlMtMCrossCurrencyBasisSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,C16,C17)</f>
-        <v>欣[test_ratehelpers.xlsx]MtMCrossCurrencyBasisSwapRateHe!R18C3MtMCrossCurrencyBasisSwapRateHelper,A</v>
+      <c r="B18" s="12" t="e">
+        <f ca="1">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13,B14,B15,B16)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C18" s="12" t="e">
+        <f ca="1">_xll.qlMtMCrossCurrencyBasisSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,C16,C17)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="12">
-        <f>_xll.qlRateHelperQuote(B18)</f>
-        <v>0.8</v>
-      </c>
-      <c r="C19" s="12">
-        <f>_xll.qlRateHelperQuote(C18)</f>
-        <v>0.8</v>
+      <c r="B19" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B18)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C19" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C18)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="11">
-        <f>_xll.qlRateHelperLatestDate(B18)</f>
-        <v>45757</v>
-      </c>
-      <c r="C20" s="11">
-        <f>_xll.qlRateHelperLatestDate(C18)</f>
-        <v>45758</v>
+      <c r="B20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B18)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C18)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B18)</f>
-        <v>45667</v>
-      </c>
-      <c r="C21" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C18)</f>
-        <v>45667</v>
+      <c r="B21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B18)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C18)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B18)</f>
-        <v>45757</v>
-      </c>
-      <c r="C22" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C18)</f>
-        <v>45757</v>
+      <c r="B22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B18)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C18)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B18)</f>
-        <v>45757</v>
-      </c>
-      <c r="C23" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C18)</f>
-        <v>45758</v>
+      <c r="B23" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B18)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C23" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C18)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="11">
-        <f>_xll.qlRateHelperPillarDate(B18)</f>
-        <v>45757</v>
-      </c>
-      <c r="C24" s="11">
-        <f>_xll.qlRateHelperPillarDate(C18)</f>
-        <v>45758</v>
+      <c r="B24" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B18)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C24" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C18)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -2308,9 +2326,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2318,7 +2336,7 @@
         <v>93</v>
       </c>
       <c r="B4" s="12">
-        <v>0.7</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2341,9 +2359,9 @@
       <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2366,27 +2384,27 @@
       <c r="A10" t="s">
         <v>168</v>
       </c>
-      <c r="B10" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]IborIborBasisSwapRateHelper!R10C2Euribor,A</v>
+      <c r="B10" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>169</v>
       </c>
-      <c r="B11" s="12" t="str">
-        <f>_xll.qlAUDLibor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]IborIborBasisSwapRateHelper!R11C2AUDLibor,A</v>
+      <c r="B11" s="12" t="e">
+        <f ca="1">_xll.qlAUDLibor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>170</v>
       </c>
-      <c r="B12" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]IborIborBasisSwapRateHelper!R12C2YieldTermStructureHandle,A</v>
+      <c r="B12" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2401,72 +2419,72 @@
       <c r="A14" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B14" s="12" t="str">
-        <f>_xll.qlIborIborBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13)</f>
-        <v>欣[test_ratehelpers.xlsx]IborIborBasisSwapRateHelper!R14C2IborIborBasisSwapRateHelper,A</v>
+      <c r="B14" s="12" t="e">
+        <f ca="1">_xll.qlIborIborBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12,B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="12">
-        <f>_xll.qlRateHelperQuote(B14)</f>
-        <v>0.7</v>
+      <c r="B15" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="11">
-        <f>_xll.qlRateHelperLatestDate(B14)</f>
-        <v>45756</v>
+      <c r="B16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B14)</f>
-        <v>45666</v>
+      <c r="B17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B14)</f>
-        <v>45756</v>
+      <c r="B18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B14)</f>
-        <v>45756</v>
+      <c r="B19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="11">
-        <f>_xll.qlRateHelperPillarDate(B14)</f>
-        <v>45756</v>
+      <c r="B20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B21" s="12" t="str">
-        <f>_xll.qlIborIborBasisSwapRateHelperSwap(B14)</f>
-        <v>欣[test_ratehelpers.xlsx]IborIborBasisSwapRateHelper!R21C2Swap,A</v>
+      <c r="B21" s="12" t="e">
+        <f ca="1">_xll.qlIborIborBasisSwapRateHelperSwap(B14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -2496,9 +2514,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2506,7 +2524,7 @@
         <v>93</v>
       </c>
       <c r="B4" s="12">
-        <v>0.3</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2529,9 +2547,9 @@
       <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="12" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B7" s="12" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2554,99 +2572,99 @@
       <c r="A10" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="12" t="str">
-        <f>_xll.qlSofr()</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIborBasisSwapRateHelpe!R10C2Sofr,A</v>
+      <c r="B10" s="12" t="e">
+        <f ca="1">_xll.qlSofr()</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>169</v>
       </c>
-      <c r="B11" s="12" t="str">
-        <f>_xll.qlAUDLibor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIborBasisSwapRateHelpe!R11C2AUDLibor,A</v>
+      <c r="B11" s="12" t="e">
+        <f ca="1">_xll.qlAUDLibor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>170</v>
       </c>
-      <c r="B12" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIborBasisSwapRateHelpe!R12C2YieldTermStructureHandle,A</v>
+      <c r="B12" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B13" s="12" t="str">
-        <f>_xll.qlOvernightIborBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12)</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIborBasisSwapRateHelpe!R13C2OvernightIborBasisSwapRateHelper,A</v>
+      <c r="B13" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIborBasisSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="12">
-        <f>_xll.qlRateHelperQuote(B13)</f>
-        <v>0.3</v>
+      <c r="B14" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="11">
-        <f>_xll.qlRateHelperLatestDate(B13)</f>
-        <v>45755</v>
+      <c r="B15" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B13)</f>
-        <v>45665</v>
+      <c r="B16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B13)</f>
-        <v>45755</v>
+      <c r="B17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B13)</f>
-        <v>45755</v>
+      <c r="B18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="11">
-        <f>_xll.qlRateHelperPillarDate(B13)</f>
-        <v>45755</v>
+      <c r="B19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B20" s="12" t="str">
-        <f>_xll.qlOvernightIborBasisSwapRateHelperSwap(B13)</f>
-        <v>欣[test_ratehelpers.xlsx]OvernightIborBasisSwapRateHelpe!R20C2Swap,A</v>
+      <c r="B20" s="12" t="e">
+        <f ca="1">_xll.qlOvernightIborBasisSwapRateHelperSwap(B13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -2678,9 +2696,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="1">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="1" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2711,9 +2729,9 @@
       <c r="A7" t="s">
         <v>60</v>
       </c>
-      <c r="B7" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]MultipleResetsSwapRateHelper!R7C2Euribor,A</v>
+      <c r="B7" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2728,9 +2746,9 @@
       <c r="A9" t="s">
         <v>46</v>
       </c>
-      <c r="B9" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]MultipleResetsSwapRateHelper!R9C2YieldTermStructureHandle,A</v>
+      <c r="B9" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -2786,9 +2804,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="1">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="1" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2798,8 +2816,8 @@
       <c r="A4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="10">
-        <v>0.2</v>
+      <c r="B4" s="18">
+        <v>0.02</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2822,9 +2840,9 @@
       <c r="A7" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B7" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2855,63 +2873,63 @@
       <c r="A11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="12" t="str">
-        <f>_xll.qlDepositRateHelper(B4,B5,B6,B7,B8,B9,B10)</f>
-        <v>欣[test_ratehelpers.xlsx]DepositRateHelper!R11C2DepositRateHelper,A</v>
+      <c r="B11" s="12" t="e">
+        <f ca="1">_xll.qlDepositRateHelper(B4,B5,B6,B7,B8,B9,B10)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="12">
-        <f>_xll.qlRateHelperQuote(B11)</f>
-        <v>0.2</v>
+      <c r="B12" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B11)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="11">
-        <f>_xll.qlRateHelperLatestDate(B11)</f>
-        <v>45754</v>
+      <c r="B13" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B11)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B11)</f>
-        <v>45663</v>
+      <c r="B14" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B11)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B11)</f>
-        <v>45754</v>
+      <c r="B15" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B11)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B11)</f>
-        <v>45754</v>
+      <c r="B16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B11)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="11">
-        <f>_xll.qlRateHelperPillarDate(B11)</f>
-        <v>45754</v>
+      <c r="B17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B11)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2924,8 +2942,8 @@
       <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="12">
-        <v>0.2</v>
+      <c r="B20" s="18">
+        <v>0.02</v>
       </c>
       <c r="E20" s="1"/>
     </row>
@@ -2933,72 +2951,72 @@
       <c r="A21" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]DepositRateHelper!R21C2Euribor,A</v>
+      <c r="B21" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="12" t="str">
-        <f>_xll.qlDepositRateHelper2(B20,B21)</f>
-        <v>欣[test_ratehelpers.xlsx]DepositRateHelper!R22C2DepositRateHelper,A</v>
+      <c r="B22" s="12" t="e">
+        <f ca="1">_xll.qlDepositRateHelper2(B20,B21)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="12">
-        <f>_xll.qlRateHelperQuote(B22)</f>
-        <v>0.2</v>
+      <c r="B23" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B22)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="11">
-        <f>_xll.qlRateHelperLatestDate(B22)</f>
-        <v>45755</v>
+      <c r="B24" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B22)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B22)</f>
-        <v>45665</v>
+      <c r="B25" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B22)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B26" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B22)</f>
-        <v>45755</v>
+      <c r="B26" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B22)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B22)</f>
-        <v>45755</v>
+      <c r="B27" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B22)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B28" s="11">
-        <f>_xll.qlRateHelperPillarDate(B22)</f>
-        <v>45755</v>
+      <c r="B28" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B22)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -3011,8 +3029,8 @@
       <c r="A31" t="s">
         <v>18</v>
       </c>
-      <c r="B31" s="12">
-        <v>0.2</v>
+      <c r="B31" s="18">
+        <v>0.02</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -3027,72 +3045,72 @@
       <c r="A33" t="s">
         <v>10</v>
       </c>
-      <c r="B33" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]DepositRateHelper!R33C2Euribor,A</v>
+      <c r="B33" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="12" t="str">
-        <f>_xll.qlDepositRateHelper3(B31,B32,B33)</f>
-        <v>欣[test_ratehelpers.xlsx]DepositRateHelper!R34C2DepositRateHelper,A</v>
+      <c r="B34" s="12" t="e">
+        <f ca="1">_xll.qlDepositRateHelper3(B31,B32,B33)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B35" s="12">
-        <f>_xll.qlRateHelperQuote(B34)</f>
-        <v>0.2</v>
+      <c r="B35" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B34)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B36" s="11">
-        <f>_xll.qlRateHelperLatestDate(B34)</f>
-        <v>45757</v>
+      <c r="B36" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B34)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B34)</f>
-        <v>45667</v>
+      <c r="B37" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B34)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B38" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B34)</f>
-        <v>45757</v>
+      <c r="B38" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B34)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B39" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B34)</f>
-        <v>45757</v>
+      <c r="B39" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B34)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="11">
-        <f>_xll.qlRateHelperPillarDate(B34)</f>
-        <v>45757</v>
+      <c r="B40" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B34)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -3125,9 +3143,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="1">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="1" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3140,13 +3158,13 @@
         <v>18</v>
       </c>
       <c r="B4" s="10">
-        <v>0.2</v>
+        <v>95.5</v>
       </c>
       <c r="C4" s="10">
-        <v>0.2</v>
+        <v>95.5</v>
       </c>
       <c r="D4" s="10">
-        <v>0.2</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3195,17 +3213,17 @@
       <c r="A8" t="s">
         <v>113</v>
       </c>
-      <c r="B8" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C8" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="D8" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B8" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C8" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D8" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3290,119 +3308,119 @@
       <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="12" t="str">
-        <f>_xll.qlFRARateHelper(B4,B5,B6,B7,B8,B9,B10,B11)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R15C2FraRateHelper,A</v>
-      </c>
-      <c r="C15" s="12" t="str">
-        <f>_xll.qlFRARateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R15C3FraRateHelper,A</v>
-      </c>
-      <c r="D15" s="12" t="str">
-        <f>_xll.qlFRARateHelper(D4,D5,D6,D7,D8,D9,D10,D11,D12,D13,D14)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R15C4FraRateHelper,A</v>
+      <c r="B15" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper(B4,B5,B6,B7,B8,B9,B10,B11)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C15" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D15" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper(D4,D5,D6,D7,D8,D9,D10,D11,D12,D13,D14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="12">
-        <f>_xll.qlRateHelperQuote(B15)</f>
-        <v>0.2</v>
-      </c>
-      <c r="C16" s="12">
-        <f>_xll.qlRateHelperQuote(C15)</f>
-        <v>0.2</v>
-      </c>
-      <c r="D16" s="12">
-        <f>_xll.qlRateHelperQuote(D15)</f>
-        <v>0.2</v>
+      <c r="B16" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C16" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D16" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(D15)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="11">
-        <f>_xll.qlRateHelperLatestDate(B15)</f>
-        <v>45846</v>
-      </c>
-      <c r="C17" s="11">
-        <f>_xll.qlRateHelperLatestDate(C15)</f>
-        <v>45816</v>
-      </c>
-      <c r="D17" s="11">
-        <f>_xll.qlRateHelperLatestDate(D15)</f>
-        <v>45816</v>
+      <c r="B17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(D15)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B15)</f>
-        <v>45665</v>
-      </c>
-      <c r="C18" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C15)</f>
-        <v>45663</v>
-      </c>
-      <c r="D18" s="11">
-        <f>_xll.qlRateHelperEarliestDate(D15)</f>
-        <v>45663</v>
+      <c r="B18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(D15)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B15)</f>
-        <v>45846</v>
-      </c>
-      <c r="C19" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C15)</f>
-        <v>45845</v>
-      </c>
-      <c r="D19" s="11">
-        <f>_xll.qlRateHelperMaturityDate(D15)</f>
-        <v>45845</v>
+      <c r="B19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(D15)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B15)</f>
-        <v>45846</v>
-      </c>
-      <c r="C20" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C15)</f>
-        <v>45845</v>
-      </c>
-      <c r="D20" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(D15)</f>
-        <v>45845</v>
+      <c r="B20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(D15)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="11">
-        <f>_xll.qlRateHelperPillarDate(B15)</f>
-        <v>45846</v>
-      </c>
-      <c r="C21" s="11">
-        <f>_xll.qlRateHelperPillarDate(C15)</f>
-        <v>45816</v>
-      </c>
-      <c r="D21" s="11">
-        <f>_xll.qlRateHelperPillarDate(D15)</f>
-        <v>45816</v>
+      <c r="B21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C15)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(D15)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3419,14 +3437,14 @@
       <c r="A24" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="12">
-        <v>0.6</v>
-      </c>
-      <c r="C24" s="12">
-        <v>0.6</v>
-      </c>
-      <c r="D24" s="12">
-        <v>0.6</v>
+      <c r="B24" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="C24" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="D24" s="10">
+        <v>95.5</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3447,17 +3465,17 @@
       <c r="A26" t="s">
         <v>115</v>
       </c>
-      <c r="B26" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R26C2Euribor,A</v>
-      </c>
-      <c r="C26" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R26C3Euribor,A</v>
-      </c>
-      <c r="D26" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R26C4Euribor,A</v>
+      <c r="B26" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C26" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D26" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3498,119 +3516,119 @@
       <c r="A30" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="12" t="str">
-        <f>_xll.qlFRARateHelper2(B24,B25,B26)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R30C2FraRateHelper,A</v>
-      </c>
-      <c r="C30" s="12" t="str">
-        <f>_xll.qlFRARateHelper2(C24,C25,C26,C27,,C29)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R30C3FraRateHelper,A</v>
-      </c>
-      <c r="D30" s="12" t="str">
-        <f>_xll.qlFRARateHelper2(D24,D25,D26,D27,D28,D29)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R30C4FraRateHelper,A</v>
+      <c r="B30" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper2(B24,B25,B26)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C30" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper2(C24,C25,C26,C27,,C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D30" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper2(D24,D25,D26,D27,D28,D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="12">
-        <f>_xll.qlRateHelperQuote(B30)</f>
-        <v>0.6</v>
-      </c>
-      <c r="C31" s="12">
-        <f>_xll.qlRateHelperQuote(C30)</f>
-        <v>0.6</v>
-      </c>
-      <c r="D31" s="12">
-        <f>_xll.qlRateHelperQuote(D30)</f>
-        <v>0.6</v>
+      <c r="B31" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C31" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D31" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(D30)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="11">
-        <f>_xll.qlRateHelperLatestDate(B30)</f>
-        <v>45755</v>
-      </c>
-      <c r="C32" s="11">
-        <f>_xll.qlRateHelperLatestDate(C30)</f>
-        <v>45755</v>
-      </c>
-      <c r="D32" s="11">
-        <f>_xll.qlRateHelperLatestDate(D30)</f>
-        <v>45724</v>
+      <c r="B32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(D30)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B33" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B30)</f>
-        <v>45665</v>
-      </c>
-      <c r="C33" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C30)</f>
-        <v>45665</v>
-      </c>
-      <c r="D33" s="11">
-        <f>_xll.qlRateHelperEarliestDate(D30)</f>
-        <v>45665</v>
+      <c r="B33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(D30)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B34" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B30)</f>
-        <v>45755</v>
-      </c>
-      <c r="C34" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C30)</f>
-        <v>45755</v>
-      </c>
-      <c r="D34" s="11">
-        <f>_xll.qlRateHelperMaturityDate(D30)</f>
-        <v>45755</v>
+      <c r="B34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(D30)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B30)</f>
-        <v>45755</v>
-      </c>
-      <c r="C35" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C30)</f>
-        <v>45755</v>
-      </c>
-      <c r="D35" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(D30)</f>
-        <v>45755</v>
+      <c r="B35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(D30)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="11">
-        <f>_xll.qlRateHelperPillarDate(B30)</f>
-        <v>45755</v>
-      </c>
-      <c r="C36" s="11">
-        <f>_xll.qlRateHelperPillarDate(C30)</f>
-        <v>45755</v>
-      </c>
-      <c r="D36" s="11">
-        <f>_xll.qlRateHelperPillarDate(D30)</f>
-        <v>45724</v>
+      <c r="B36" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C36" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C30)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D36" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(D30)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -3627,14 +3645,14 @@
       <c r="A39" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="12">
-        <v>0.33</v>
-      </c>
-      <c r="C39" s="12">
-        <v>0.33</v>
-      </c>
-      <c r="D39" s="12">
-        <v>0.33</v>
+      <c r="B39" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="C39" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="D39" s="10">
+        <v>95.5</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -3669,17 +3687,17 @@
       <c r="A42" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B42" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R42C2Euribor,A</v>
-      </c>
-      <c r="C42" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R42C3Euribor,A</v>
-      </c>
-      <c r="D42" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R42C4Euribor,A</v>
+      <c r="B42" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C42" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D42" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -3720,119 +3738,119 @@
       <c r="A46" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B46" s="12" t="str">
-        <f>_xll.qlFRARateHelper3(B39,B40,B41,B42)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R46C2FraRateHelper,A</v>
-      </c>
-      <c r="C46" s="12" t="str">
-        <f>_xll.qlFRARateHelper3(C39,C40,C41,C42,C43,,C45)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R46C3FraRateHelper,A</v>
-      </c>
-      <c r="D46" s="12" t="str">
-        <f>_xll.qlFRARateHelper3(D39,D40,D41,D42,D43,D44,D45)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R46C4FraRateHelper,A</v>
+      <c r="B46" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper3(B39,B40,B41,B42)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C46" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper3(C39,C40,C41,C42,C43,,C45)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D46" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper3(D39,D40,D41,D42,D43,D44,D45)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B47" s="12">
-        <f>_xll.qlRateHelperQuote(B46)</f>
-        <v>0.33</v>
-      </c>
-      <c r="C47" s="12">
-        <f>_xll.qlRateHelperQuote(C46)</f>
-        <v>0.33</v>
-      </c>
-      <c r="D47" s="12">
-        <f>_xll.qlRateHelperQuote(D46)</f>
-        <v>0.33</v>
+      <c r="B47" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C47" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D47" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(D46)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B48" s="11">
-        <f>_xll.qlRateHelperLatestDate(B46)</f>
-        <v>45918</v>
-      </c>
-      <c r="C48" s="11">
-        <f>_xll.qlRateHelperLatestDate(C46)</f>
-        <v>45917</v>
-      </c>
-      <c r="D48" s="11">
-        <f>_xll.qlRateHelperLatestDate(D46)</f>
-        <v>45846</v>
+      <c r="B48" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C48" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D48" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(D46)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B49" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B46)</f>
-        <v>45826</v>
-      </c>
-      <c r="C49" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C46)</f>
-        <v>45826</v>
-      </c>
-      <c r="D49" s="11">
-        <f>_xll.qlRateHelperEarliestDate(D46)</f>
-        <v>45826</v>
+      <c r="B49" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C49" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D49" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(D46)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B50" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B46)</f>
-        <v>45917</v>
-      </c>
-      <c r="C50" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C46)</f>
-        <v>45917</v>
-      </c>
-      <c r="D50" s="11">
-        <f>_xll.qlRateHelperMaturityDate(D46)</f>
-        <v>45917</v>
+      <c r="B50" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C50" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D50" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(D46)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B51" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B46)</f>
-        <v>45918</v>
-      </c>
-      <c r="C51" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C46)</f>
-        <v>45918</v>
-      </c>
-      <c r="D51" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(D46)</f>
-        <v>45918</v>
+      <c r="B51" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C51" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D51" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(D46)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B52" s="11">
-        <f>_xll.qlRateHelperPillarDate(B46)</f>
-        <v>45918</v>
-      </c>
-      <c r="C52" s="11">
-        <f>_xll.qlRateHelperPillarDate(C46)</f>
-        <v>45917</v>
-      </c>
-      <c r="D52" s="11">
-        <f>_xll.qlRateHelperPillarDate(D46)</f>
-        <v>45846</v>
+      <c r="B52" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C52" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C46)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D52" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(D46)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -3849,14 +3867,14 @@
       <c r="A55" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B55" s="12">
-        <v>0.44</v>
-      </c>
-      <c r="C55" s="12">
-        <v>0.44</v>
-      </c>
-      <c r="D55" s="12">
-        <v>0.44</v>
+      <c r="B55" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="C55" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="D55" s="10">
+        <v>95.5</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -3877,17 +3895,17 @@
       <c r="A57" t="s">
         <v>25</v>
       </c>
-      <c r="B57" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R57C2Euribor,A</v>
-      </c>
-      <c r="C57" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R57C3Euribor,A</v>
-      </c>
-      <c r="D57" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R57C4Euribor,A</v>
+      <c r="B57" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C57" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D57" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -3928,119 +3946,119 @@
       <c r="A61" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B61" s="12" t="str">
-        <f>_xll.qlFRARateHelper4(B55,B56,B57)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R61C2FraRateHelper,A</v>
-      </c>
-      <c r="C61" s="12" t="str">
-        <f>_xll.qlFRARateHelper4(C55,C56,C57,C58,,C60)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R61C3FraRateHelper,A</v>
-      </c>
-      <c r="D61" s="12" t="str">
-        <f>_xll.qlFRARateHelper4(D55,D56,D57,D58,D59,D60)</f>
-        <v>欣[test_ratehelpers.xlsx]FRARateHelper!R61C4FraRateHelper,A</v>
+      <c r="B61" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper4(B55,B56,B57)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C61" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper4(C55,C56,C57,C58,,C60)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D61" s="12" t="e">
+        <f ca="1">_xll.qlFRARateHelper4(D55,D56,D57,D58,D59,D60)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B62" s="12">
-        <f>_xll.qlRateHelperQuote(B61)</f>
-        <v>0.44</v>
-      </c>
-      <c r="C62" s="12">
-        <f>_xll.qlRateHelperQuote(C61)</f>
-        <v>0.44</v>
-      </c>
-      <c r="D62" s="12">
-        <f>_xll.qlRateHelperQuote(D61)</f>
-        <v>0.44</v>
+      <c r="B62" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C62" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D62" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(D61)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B63" s="11">
-        <f>_xll.qlRateHelperLatestDate(B61)</f>
-        <v>45938</v>
-      </c>
-      <c r="C63" s="11">
-        <f>_xll.qlRateHelperLatestDate(C61)</f>
-        <v>45938</v>
-      </c>
-      <c r="D63" s="11">
-        <f>_xll.qlRateHelperLatestDate(D61)</f>
-        <v>45846</v>
+      <c r="B63" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C63" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D63" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(D61)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B64" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B61)</f>
-        <v>45846</v>
-      </c>
-      <c r="C64" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C61)</f>
-        <v>45846</v>
-      </c>
-      <c r="D64" s="11">
-        <f>_xll.qlRateHelperEarliestDate(D61)</f>
-        <v>45846</v>
+      <c r="B64" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C64" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D64" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(D61)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B65" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B61)</f>
-        <v>45938</v>
-      </c>
-      <c r="C65" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C61)</f>
-        <v>45938</v>
-      </c>
-      <c r="D65" s="11">
-        <f>_xll.qlRateHelperMaturityDate(D61)</f>
-        <v>45938</v>
+      <c r="B65" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C65" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D65" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(D61)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B66" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B61)</f>
-        <v>45938</v>
-      </c>
-      <c r="C66" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C61)</f>
-        <v>45938</v>
-      </c>
-      <c r="D66" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(D61)</f>
-        <v>45938</v>
+      <c r="B66" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C66" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D66" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(D61)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B67" s="11">
-        <f>_xll.qlRateHelperPillarDate(B61)</f>
-        <v>45938</v>
-      </c>
-      <c r="C67" s="11">
-        <f>_xll.qlRateHelperPillarDate(C61)</f>
-        <v>45938</v>
-      </c>
-      <c r="D67" s="11">
-        <f>_xll.qlRateHelperPillarDate(D61)</f>
-        <v>45846</v>
+      <c r="B67" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C67" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C61)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D67" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(D61)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -4055,7 +4073,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.85546875" customWidth="1"/>
-    <col min="2" max="2" width="64.28515625" customWidth="1"/>
+    <col min="2" max="2" width="104.5703125" customWidth="1"/>
     <col min="3" max="3" width="69" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4072,9 +4090,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="1">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="1" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -4086,10 +4104,10 @@
         <v>116</v>
       </c>
       <c r="B4" s="10">
-        <v>0.4</v>
+        <v>95.5</v>
       </c>
       <c r="C4" s="10">
-        <v>0.4</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4118,13 +4136,13 @@
       <c r="A7" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C7" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B7" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -4182,104 +4200,104 @@
       <c r="A13" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="12" t="str">
-        <f>_xll.qlFuturesRateHelper(B4,B5,B6,B7,B8,B9,B10)</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R13C2FuturesRateHelper,A</v>
-      </c>
-      <c r="C13" s="12" t="str">
-        <f>_xll.qlFuturesRateHelper(C4,C5,C6,C7,C8,C9,C10,,C12)</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R13C3FuturesRateHelper,A</v>
+      <c r="B13" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateHelper(B4,B5,B6,B7,B8,B9,B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C13" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateHelper(C4,C5,C6,C7,C8,C9,C10,,C12)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="12">
-        <f>_xll.qlRateHelperQuote(B13)</f>
-        <v>0.4</v>
-      </c>
-      <c r="C14" s="12">
-        <f>_xll.qlRateHelperQuote(C13)</f>
-        <v>0.4</v>
+      <c r="B14" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C14" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="11">
-        <f>_xll.qlRateHelperLatestDate(B13)</f>
-        <v>45918</v>
-      </c>
-      <c r="C15" s="11">
-        <f>_xll.qlRateHelperLatestDate(C13)</f>
-        <v>45950</v>
+      <c r="B15" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C15" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B13)</f>
-        <v>45826</v>
-      </c>
-      <c r="C16" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C13)</f>
-        <v>45826</v>
+      <c r="B16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B13)</f>
-        <v>45918</v>
-      </c>
-      <c r="C17" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C13)</f>
-        <v>45950</v>
+      <c r="B17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B13)</f>
-        <v>45918</v>
-      </c>
-      <c r="C18" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C13)</f>
-        <v>45950</v>
+      <c r="B18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="11">
-        <f>_xll.qlRateHelperPillarDate(B13)</f>
-        <v>45918</v>
-      </c>
-      <c r="C19" s="11">
-        <f>_xll.qlRateHelperPillarDate(C13)</f>
-        <v>45950</v>
+      <c r="B19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="12">
-        <f>_xll.qlFuturesRateConvexityAdjustment(B13)</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="12">
-        <f>_xll.qlFuturesRateConvexityAdjustment(C13)</f>
-        <v>0</v>
+      <c r="B20" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateConvexityAdjustment(B13)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateConvexityAdjustment(C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -4292,11 +4310,11 @@
       <c r="A23" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B23" s="12">
-        <v>0.3</v>
-      </c>
-      <c r="C23" s="12">
-        <v>0.3</v>
+      <c r="B23" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="C23" s="10">
+        <v>95.5</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -4354,115 +4372,115 @@
       <c r="A29" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B29" t="str">
-        <f>_xll.qlFuturesRateHelper2(B23,B24,B25,B26)</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R29C2FuturesRateHelper,A</v>
-      </c>
-      <c r="C29" t="str">
-        <f>_xll.qlFuturesRateHelper2(C23,C24,C25,C26,,C28)</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R29C3FuturesRateHelper,A</v>
+      <c r="B29" t="e">
+        <f ca="1">_xll.qlFuturesRateHelper2(B23,B24,B25,B26)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C29" t="e">
+        <f ca="1">_xll.qlFuturesRateHelper2(C23,C24,C25,C26,,C28)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="12">
-        <f>_xll.qlRateHelperQuote(B29)</f>
-        <v>0.3</v>
-      </c>
-      <c r="C30" s="12">
-        <f>_xll.qlRateHelperQuote(C29)</f>
-        <v>0.3</v>
+      <c r="B30" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C30" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="11">
-        <f>_xll.qlRateHelperLatestDate(B29)</f>
-        <v>45917</v>
-      </c>
-      <c r="C31" s="11">
-        <f>_xll.qlRateHelperLatestDate(C29)</f>
-        <v>45917</v>
+      <c r="B31" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C31" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B29)</f>
-        <v>45826</v>
-      </c>
-      <c r="C32" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C29)</f>
-        <v>45826</v>
+      <c r="B32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B29)</f>
-        <v>45917</v>
-      </c>
-      <c r="C33" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C29)</f>
-        <v>45917</v>
+      <c r="B33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B29)</f>
-        <v>45917</v>
-      </c>
-      <c r="C34" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C29)</f>
-        <v>45917</v>
+      <c r="B34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="11">
-        <f>_xll.qlRateHelperPillarDate(B29)</f>
-        <v>45917</v>
-      </c>
-      <c r="C35" s="11">
-        <f>_xll.qlRateHelperPillarDate(C29)</f>
-        <v>45917</v>
+      <c r="B35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B36" s="12">
-        <f>_xll.qlFuturesRateConvexityAdjustment(B29)</f>
-        <v>0</v>
-      </c>
-      <c r="C36" s="12">
-        <f>_xll.qlFuturesRateConvexityAdjustment(C29)</f>
-        <v>0</v>
+      <c r="B36" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateConvexityAdjustment(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C36" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateConvexityAdjustment(C29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B39" s="12">
-        <v>0.33</v>
-      </c>
-      <c r="C39" s="12">
-        <v>0.33</v>
+      <c r="B39" s="10">
+        <v>95.5</v>
+      </c>
+      <c r="C39" s="10">
+        <v>95.5</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -4480,13 +4498,13 @@
       <c r="A41" t="s">
         <v>124</v>
       </c>
-      <c r="B41" s="12" t="str">
-        <f>_xll.qlEuribor("6M")</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R41C2Euribor,A</v>
-      </c>
-      <c r="C41" s="12" t="str">
-        <f>_xll.qlEuribor("6M")</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R41C3Euribor,A</v>
+      <c r="B41" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("6M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C41" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("6M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -4511,104 +4529,104 @@
       <c r="A44" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B44" t="str">
-        <f>_xll.qlFuturesRateHelper3(B39,B40,B41)</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R44C2FuturesRateHelper,A</v>
-      </c>
-      <c r="C44" t="str">
-        <f>_xll.qlFuturesRateHelper3(C39,C40,C41,,C43)</f>
-        <v>欣[test_ratehelpers.xlsx]FutureRateHelper!R44C3FuturesRateHelper,A</v>
+      <c r="B44" t="e">
+        <f ca="1">_xll.qlFuturesRateHelper3(B39,B40,B41)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C44" t="e">
+        <f ca="1">_xll.qlFuturesRateHelper3(C39,C40,C41,,C43)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B45" s="12">
-        <f>_xll.qlRateHelperQuote(B44)</f>
-        <v>0.33</v>
-      </c>
-      <c r="C45" s="12">
-        <f>_xll.qlRateHelperQuote(C44)</f>
-        <v>0.33</v>
+      <c r="B45" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C45" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C44)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B46" s="11">
-        <f>_xll.qlRateHelperLatestDate(B44)</f>
-        <v>46009</v>
-      </c>
-      <c r="C46" s="11">
-        <f>_xll.qlRateHelperLatestDate(C44)</f>
-        <v>46009</v>
+      <c r="B46" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C46" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C44)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B47" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B44)</f>
-        <v>45826</v>
-      </c>
-      <c r="C47" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C44)</f>
-        <v>45826</v>
+      <c r="B47" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C47" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C44)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B48" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B44)</f>
-        <v>46009</v>
-      </c>
-      <c r="C48" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C44)</f>
-        <v>46009</v>
+      <c r="B48" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C48" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C44)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B49" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B44)</f>
-        <v>46009</v>
-      </c>
-      <c r="C49" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C44)</f>
-        <v>46009</v>
+      <c r="B49" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C49" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C44)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B50" s="11">
-        <f>_xll.qlRateHelperPillarDate(B44)</f>
-        <v>46009</v>
-      </c>
-      <c r="C50" s="11">
-        <f>_xll.qlRateHelperPillarDate(C44)</f>
-        <v>46009</v>
+      <c r="B50" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C50" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C44)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="12">
-        <f>_xll.qlFuturesRateConvexityAdjustment(B44)</f>
-        <v>0</v>
-      </c>
-      <c r="C51" s="12">
-        <f>_xll.qlFuturesRateConvexityAdjustment(C44)</f>
-        <v>0</v>
+      <c r="B51" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateConvexityAdjustment(B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C51" s="12" t="e">
+        <f ca="1">_xll.qlFuturesRateConvexityAdjustment(C44)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -4638,9 +4656,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -4654,14 +4672,14 @@
       <c r="A4" t="s">
         <v>125</v>
       </c>
-      <c r="B4" s="10">
-        <v>0.4</v>
-      </c>
-      <c r="C4" s="10">
-        <v>0.4</v>
-      </c>
-      <c r="D4" s="10">
-        <v>0.4</v>
+      <c r="B4" s="18">
+        <v>0.04</v>
+      </c>
+      <c r="C4" s="18">
+        <v>0.04</v>
+      </c>
+      <c r="D4" s="18">
+        <v>0.04</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
@@ -4686,17 +4704,17 @@
       <c r="A6" t="s">
         <v>113</v>
       </c>
-      <c r="B6" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C6" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="D6" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B6" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C6" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D6" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -4753,17 +4771,17 @@
       <c r="A10" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R10C2Euribor,A</v>
-      </c>
-      <c r="C10" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R10C3Euribor,A</v>
-      </c>
-      <c r="D10" s="12" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R10C4Euribor,A</v>
+      <c r="B10" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C10" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D10" s="12" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
@@ -4801,13 +4819,13 @@
         <v>153</v>
       </c>
       <c r="B13" s="11"/>
-      <c r="C13" s="11" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R13C3YieldTermStructureHandle,A</v>
-      </c>
-      <c r="D13" s="11" t="str">
-        <f>_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R13C4YieldTermStructureHandle,A</v>
+      <c r="C13" s="11" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D13" s="11" t="e">
+        <f ca="1">_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
@@ -4884,153 +4902,153 @@
       <c r="A19" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="12" t="str">
-        <f>_xll.qlSwapRateHelper(B4,B5,B6,B7,B8,B9,B10)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R19C2SwapRateHelper,A</v>
-      </c>
-      <c r="C19" s="12" t="str">
-        <f>_xll.qlSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,,C17,C18)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R19C3SwapRateHelper,A</v>
-      </c>
-      <c r="D19" s="12" t="str">
-        <f>_xll.qlSwapRateHelper(D4,D5,D6,D7,D8,D9,D10,D11,D12,D13,D14,D15,D16,D17,D18)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R19C4SwapRateHelper,A</v>
+      <c r="B19" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelper(B4,B5,B6,B7,B8,B9,B10)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C19" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,,C17,C18)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D19" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelper(D4,D5,D6,D7,D8,D9,D10,D11,D12,D13,D14,D15,D16,D17,D18)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="12">
-        <f>_xll.qlRateHelperQuote(B19)</f>
-        <v>0.4</v>
-      </c>
-      <c r="C20" s="12">
-        <f>_xll.qlRateHelperQuote(C19)</f>
-        <v>0.4</v>
-      </c>
-      <c r="D20" s="12">
-        <f>_xll.qlRateHelperQuote(D19)</f>
-        <v>0.4</v>
+      <c r="B20" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D20" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="11">
-        <f>_xll.qlRateHelperLatestDate(B19)</f>
-        <v>45754</v>
-      </c>
-      <c r="C21" s="11">
-        <f>_xll.qlRateHelperLatestDate(C19)</f>
-        <v>45846</v>
-      </c>
-      <c r="D21" s="11">
-        <f>_xll.qlRateHelperLatestDate(D19)</f>
-        <v>45784</v>
+      <c r="B21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D21" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B19)</f>
-        <v>45663</v>
-      </c>
-      <c r="C22" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C19)</f>
-        <v>45755</v>
-      </c>
-      <c r="D22" s="11">
-        <f>_xll.qlRateHelperEarliestDate(D19)</f>
-        <v>45755</v>
+      <c r="B22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D22" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B19)</f>
-        <v>45754</v>
-      </c>
-      <c r="C23" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C19)</f>
-        <v>45846</v>
-      </c>
-      <c r="D23" s="11">
-        <f>_xll.qlRateHelperMaturityDate(D19)</f>
-        <v>45846</v>
+      <c r="B23" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C23" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D23" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B19)</f>
-        <v>45754</v>
-      </c>
-      <c r="C24" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C19)</f>
-        <v>45846</v>
-      </c>
-      <c r="D24" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(D19)</f>
-        <v>45846</v>
+      <c r="B24" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C24" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D24" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="11">
-        <f>_xll.qlRateHelperPillarDate(B19)</f>
-        <v>45754</v>
-      </c>
-      <c r="C25" s="11">
-        <f>_xll.qlRateHelperPillarDate(C19)</f>
-        <v>45846</v>
-      </c>
-      <c r="D25" s="11">
-        <f>_xll.qlRateHelperPillarDate(D19)</f>
-        <v>45784</v>
+      <c r="B25" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C25" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D25" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="12">
-        <f>_xll.qlSwapRateHelperSpread(B19)</f>
-        <v>0</v>
-      </c>
-      <c r="C26" s="12">
-        <f>_xll.qlSwapRateHelperSpread(C19)</f>
-        <v>0.5</v>
-      </c>
-      <c r="D26" s="12">
-        <f>_xll.qlSwapRateHelperSpread(D19)</f>
-        <v>0.5</v>
+      <c r="B26" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSpread(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C26" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSpread(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D26" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSpread(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="12" t="str">
-        <f>_xll.qlSwapRateHelperSwap(B19)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R27C2VanillaSwap,A</v>
-      </c>
-      <c r="C27" s="12" t="str">
-        <f>_xll.qlSwapRateHelperSwap(C19)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R27C3VanillaSwap,A</v>
-      </c>
-      <c r="D27" s="12" t="str">
-        <f>_xll.qlSwapRateHelperSwap(D19)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R27C4VanillaSwap,A</v>
+      <c r="B27" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSwap(B19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C27" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSwap(C19)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D27" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSwap(D19)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -5099,17 +5117,17 @@
       <c r="A34" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B34" s="14" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C34" s="14" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="D34" s="14" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B34" s="14" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C34" s="14" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D34" s="14" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
@@ -5158,65 +5176,65 @@
       <c r="A38" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B38" s="14" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R38C2Euribor,A</v>
-      </c>
-      <c r="C38" s="14" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R38C3Euribor,A</v>
-      </c>
-      <c r="D38" s="14" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R38C4Euribor,A</v>
+      <c r="B38" s="14" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C38" s="14" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D38" s="14" t="e">
+        <f ca="1">_xll.qlEuribor("3M")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B39" s="14" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R39C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C39" s="14" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R39C3YieldTermStructureHandle,A</v>
-      </c>
-      <c r="D39" s="14" t="str">
-        <f>_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R39C4YieldTermStructureHandle,A</v>
+      <c r="B39" s="14" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C39" s="14" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D39" s="14" t="e">
+        <f ca="1">_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B40" s="12">
-        <v>0.4</v>
-      </c>
-      <c r="C40" s="12">
-        <v>0.4</v>
-      </c>
-      <c r="D40" s="12">
-        <v>0.4</v>
+      <c r="B40" s="18">
+        <v>0.04</v>
+      </c>
+      <c r="C40" s="18">
+        <v>0.04</v>
+      </c>
+      <c r="D40" s="18">
+        <v>0.04</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B41" s="12" t="str">
-        <f>_xll.qlSwapIndex(B30,B31,B32,B33,B34,B35,B36,B37,B38,B39)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R41C2SwapIndex,A</v>
-      </c>
-      <c r="C41" s="12" t="str">
-        <f>_xll.qlSwapIndex(C30,C31,C32,C33,C34,C35,C36,C37,C38,C39)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R41C3SwapIndex,A</v>
-      </c>
-      <c r="D41" s="12" t="str">
-        <f>_xll.qlSwapIndex(D30,D31,D32,D33,D34,D35,D36,D37,D38,D39)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R41C4SwapIndex,A</v>
+      <c r="B41" s="12" t="e">
+        <f ca="1">_xll.qlSwapIndex(B30,B31,B32,B33,B34,B35,B36,B37,B38,B39)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C41" s="12" t="e">
+        <f ca="1">_xll.qlSwapIndex(C30,C31,C32,C33,C34,C35,C36,C37,C38,C39)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D41" s="12" t="e">
+        <f ca="1">_xll.qlSwapIndex(D30,D31,D32,D33,D34,D35,D36,D37,D38,D39)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -5245,13 +5263,13 @@
       <c r="A44" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C44" s="12" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R44C3YieldTermStructureHandle,A</v>
-      </c>
-      <c r="D44" s="12" t="str">
-        <f>_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R44C4YieldTermStructureHandle,A</v>
+      <c r="C44" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D44" s="12" t="e">
+        <f ca="1">_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -5299,153 +5317,153 @@
       <c r="A49" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B49" s="12" t="str">
-        <f>_xll.qlSwapRateHelper2(B40,B41)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R49C2SwapRateHelper,A</v>
-      </c>
-      <c r="C49" s="12" t="str">
-        <f>_xll.qlSwapRateHelper2(C40,C41,C42,C43,C44,C45,,C47,C48)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R49C3SwapRateHelper,A</v>
-      </c>
-      <c r="D49" s="12" t="str">
-        <f>_xll.qlSwapRateHelper2(D40,D41,D42,D43,D44,D45,D46,D47,D48)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R49C4SwapRateHelper,A</v>
+      <c r="B49" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelper2(B40,B41)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C49" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelper2(C40,C41,C42,C43,C44,C45,,C47,C48)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D49" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelper2(D40,D41,D42,D43,D44,D45,D46,D47,D48)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B50" s="12">
-        <f>_xll.qlRateHelperQuote(B49)</f>
-        <v>0.4</v>
-      </c>
-      <c r="C50" s="12">
-        <f>_xll.qlRateHelperQuote(C49)</f>
-        <v>0.4</v>
-      </c>
-      <c r="D50" s="12">
-        <f>_xll.qlRateHelperQuote(D49)</f>
-        <v>0.4</v>
+      <c r="B50" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C50" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D50" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="11">
-        <f>_xll.qlRateHelperLatestDate(B49)</f>
-        <v>45755</v>
-      </c>
-      <c r="C51" s="11">
-        <f>_xll.qlRateHelperLatestDate(C49)</f>
-        <v>45789</v>
-      </c>
-      <c r="D51" s="11">
-        <f>_xll.qlRateHelperLatestDate(D49)</f>
-        <v>45784</v>
+      <c r="B51" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C51" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D51" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B52" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B49)</f>
-        <v>45665</v>
-      </c>
-      <c r="C52" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C49)</f>
-        <v>45698</v>
-      </c>
-      <c r="D52" s="11">
-        <f>_xll.qlRateHelperEarliestDate(D49)</f>
-        <v>45698</v>
+      <c r="B52" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C52" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D52" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B53" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B49)</f>
-        <v>45755</v>
-      </c>
-      <c r="C53" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C49)</f>
-        <v>45789</v>
-      </c>
-      <c r="D53" s="11">
-        <f>_xll.qlRateHelperMaturityDate(D49)</f>
-        <v>45789</v>
+      <c r="B53" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C53" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D53" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B49)</f>
-        <v>45755</v>
-      </c>
-      <c r="C54" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C49)</f>
-        <v>45789</v>
-      </c>
-      <c r="D54" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(D49)</f>
-        <v>45789</v>
+      <c r="B54" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C54" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D54" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B55" s="11">
-        <f>_xll.qlRateHelperPillarDate(B49)</f>
-        <v>45755</v>
-      </c>
-      <c r="C55" s="11">
-        <f>_xll.qlRateHelperPillarDate(C49)</f>
-        <v>45789</v>
-      </c>
-      <c r="D55" s="11">
-        <f>_xll.qlRateHelperPillarDate(D49)</f>
-        <v>45784</v>
+      <c r="B55" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C55" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D55" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B56" s="12">
-        <f>_xll.qlSwapRateHelperSpread(B49)</f>
-        <v>0</v>
-      </c>
-      <c r="C56" s="12">
-        <f>_xll.qlSwapRateHelperSpread(C49)</f>
-        <v>0.6</v>
-      </c>
-      <c r="D56" s="12">
-        <f>_xll.qlSwapRateHelperSpread(D49)</f>
-        <v>0.6</v>
+      <c r="B56" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSpread(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C56" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSpread(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D56" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSpread(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B57" s="12" t="str">
-        <f>_xll.qlSwapRateHelperSwap(B49)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R57C2VanillaSwap,A</v>
-      </c>
-      <c r="C57" s="12" t="str">
-        <f>_xll.qlSwapRateHelperSwap(C49)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R57C3VanillaSwap,A</v>
-      </c>
-      <c r="D57" s="12" t="str">
-        <f>_xll.qlSwapRateHelperSwap(D49)</f>
-        <v>欣[test_ratehelpers.xlsx]SwapRateHelper!R57C4VanillaSwap,A</v>
+      <c r="B57" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSwap(B49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C57" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSwap(C49)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D57" s="12" t="e">
+        <f ca="1">_xll.qlSwapRateHelperSwap(D49)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -5534,9 +5552,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -5574,31 +5592,31 @@
       <c r="A6" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="10">
-        <v>0.6</v>
-      </c>
-      <c r="C6" s="10">
-        <v>0.6</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0.6</v>
+      <c r="B6" s="19">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="C6" s="19">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="D6" s="19">
+        <v>4.4999999999999998E-2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>142</v>
       </c>
-      <c r="B7" s="11" t="str">
-        <f>_xll.qlSofr()</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R7C2Sofr,A</v>
-      </c>
-      <c r="C7" s="11" t="str">
-        <f>_xll.qlSofr()</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R7C3Sofr,A</v>
-      </c>
-      <c r="D7" s="11" t="str">
-        <f>_xll.qlSofr()</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R7C4Sofr,A</v>
+      <c r="B7" s="11" t="e">
+        <f ca="1">_xll.qlSofr()</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="11" t="e">
+        <f ca="1">_xll.qlSofr()</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D7" s="11" t="e">
+        <f ca="1">_xll.qlSofr()</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -5606,13 +5624,13 @@
         <v>153</v>
       </c>
       <c r="B8" s="11"/>
-      <c r="C8" s="11" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R8C3YieldTermStructureHandle,A</v>
-      </c>
-      <c r="D8" s="11" t="str">
-        <f>_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R8C4YieldTermStructureHandle,A</v>
+      <c r="C8" s="11" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D8" s="11" t="e">
+        <f ca="1">_xll.qlFlatForward(C1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -5668,13 +5686,13 @@
         <v>154</v>
       </c>
       <c r="B13" s="11"/>
-      <c r="C13" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="D13" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="C13" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D13" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -5764,13 +5782,13 @@
         <v>156</v>
       </c>
       <c r="B21" s="11"/>
-      <c r="C21" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="D21" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="C21" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D21" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -5834,13 +5852,13 @@
         <v>158</v>
       </c>
       <c r="B27" s="11"/>
-      <c r="C27" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="D27" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="C27" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D27" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -5859,136 +5877,136 @@
       <c r="A29" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="12" t="str">
-        <f>_xll.qlOISRateHelper(B4,B5,B6,B7)</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R29C2OISRateHelper,A</v>
-      </c>
-      <c r="C29" s="12" t="str">
-        <f>_xll.qlOISRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,C16,,C18,C19,C20,C21,C22,C23,C24,,C26,C27,C28)</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R29C3OISRateHelper,A</v>
-      </c>
-      <c r="D29" s="12" t="str">
-        <f>_xll.qlOISRateHelper(D4,D5,D6,D7,D8,D9,D10,D11,D12,D13,D14,D15,D16,D17,D18,D19,D20,D21,D22,D23,D24,,D26,D27,D28)</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R29C4OISRateHelper,A</v>
+      <c r="B29" s="12" t="e">
+        <f ca="1">_xll.qlOISRateHelper(B4,B5,B6,B7)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C29" s="12" t="e">
+        <f ca="1">_xll.qlOISRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13,C14,C15,C16,,C18,C19,C20,C21,C22,C23,C24,,C26,C27,C28)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D29" s="12" t="e">
+        <f ca="1">_xll.qlOISRateHelper(D4,D5,D6,D7,D8,D9,D10,D11,D12,D13,D14,D15,D16,D17,D18,D19,D20,D21,D22,D23,D24,,D26,D27,D28)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="12">
-        <f>_xll.qlRateHelperQuote(B29)</f>
-        <v>0.6</v>
-      </c>
-      <c r="C30" s="12">
-        <f>_xll.qlRateHelperQuote(C29)</f>
-        <v>0.6</v>
-      </c>
-      <c r="D30" s="12">
-        <f>_xll.qlRateHelperQuote(D29)</f>
-        <v>0.6</v>
+      <c r="B30" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C30" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D30" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="11">
-        <f>_xll.qlRateHelperLatestDate(B29)</f>
-        <v>45756</v>
-      </c>
-      <c r="C31" s="11">
-        <f>_xll.qlRateHelperLatestDate(C29)</f>
-        <v>45791</v>
-      </c>
-      <c r="D31" s="11">
-        <f>_xll.qlRateHelperLatestDate(D29)</f>
-        <v>45791</v>
+      <c r="B31" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C31" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D31" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B29)</f>
-        <v>45666</v>
-      </c>
-      <c r="C32" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C29)</f>
-        <v>45698</v>
-      </c>
-      <c r="D32" s="11">
-        <f>_xll.qlRateHelperEarliestDate(D29)</f>
-        <v>45698</v>
+      <c r="B32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D32" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B29)</f>
-        <v>45756</v>
-      </c>
-      <c r="C33" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C29)</f>
-        <v>45789</v>
-      </c>
-      <c r="D33" s="11">
-        <f>_xll.qlRateHelperMaturityDate(D29)</f>
-        <v>45789</v>
+      <c r="B33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D33" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B29)</f>
-        <v>45756</v>
-      </c>
-      <c r="C34" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C29)</f>
-        <v>45791</v>
-      </c>
-      <c r="D34" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(D29)</f>
-        <v>45791</v>
+      <c r="B34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D34" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="11">
-        <f>_xll.qlRateHelperPillarDate(B29)</f>
-        <v>45756</v>
-      </c>
-      <c r="C35" s="11">
-        <f>_xll.qlRateHelperPillarDate(C29)</f>
-        <v>45789</v>
-      </c>
-      <c r="D35" s="11">
-        <f>_xll.qlRateHelperPillarDate(D29)</f>
-        <v>45784</v>
+      <c r="B35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D35" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B36" s="12" t="str">
-        <f>_xll.qlOISRateHelperSwap(B29)</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R36C2OvernightIndexedSwap,A</v>
-      </c>
-      <c r="C36" s="12" t="str">
-        <f>_xll.qlOISRateHelperSwap(C29)</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R36C3OvernightIndexedSwap,A</v>
-      </c>
-      <c r="D36" s="12" t="str">
-        <f>_xll.qlOISRateHelperSwap(D29)</f>
-        <v>欣[test_ratehelpers.xlsx]OISRateHelper!R36C4OvernightIndexedSwap,A</v>
+      <c r="B36" s="12" t="e">
+        <f ca="1">_xll.qlOISRateHelperSwap(B29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C36" s="12" t="e">
+        <f ca="1">_xll.qlOISRateHelperSwap(C29)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D36" s="12" t="e">
+        <f ca="1">_xll.qlOISRateHelperSwap(D29)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -6019,9 +6037,9 @@
       <c r="A2" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="11">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45663</v>
+      <c r="B2" s="11" t="e">
+        <f ca="1">_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -6032,10 +6050,10 @@
         <v>66</v>
       </c>
       <c r="B4" s="10">
-        <v>0.3</v>
+        <v>1E-3</v>
       </c>
       <c r="C4" s="10">
-        <v>0.3</v>
+        <v>1E-3</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -6043,10 +6061,10 @@
         <v>67</v>
       </c>
       <c r="B5" s="10">
-        <v>0.5</v>
+        <v>0.97</v>
       </c>
       <c r="C5" s="10">
-        <v>0.5</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -6075,13 +6093,13 @@
       <c r="A8" t="s">
         <v>113</v>
       </c>
-      <c r="B8" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C8" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="B8" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C8" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -6121,13 +6139,13 @@
       <c r="A12" t="s">
         <v>162</v>
       </c>
-      <c r="B12" s="11" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]FXSwapRateHelper!R12C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C12" s="11" t="str">
-        <f>_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
-        <v>欣[test_ratehelpers.xlsx]FXSwapRateHelper!R12C3YieldTermStructureHandle,A</v>
+      <c r="B12" s="11" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C12" s="11" t="e">
+        <f ca="1">_xll.qlFlatForward(B1,0.03,"Actual360","Compounded","Annual")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -6135,217 +6153,217 @@
         <v>161</v>
       </c>
       <c r="B13" s="11"/>
-      <c r="C13" s="11" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
+      <c r="C13" s="11" t="e">
+        <f ca="1">_xll.qlCalendar("TARGET")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12)</f>
-        <v>欣[test_ratehelpers.xlsx]FXSwapRateHelper!R14C2FxSwapRateHelper,A</v>
-      </c>
-      <c r="C14" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13)</f>
-        <v>欣[test_ratehelpers.xlsx]FXSwapRateHelper!R14C3FxSwapRateHelper,A</v>
+      <c r="B14" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelper(B4,B5,B6,B7,B8,B9,B10,B11,B12)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C14" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelper(C4,C5,C6,C7,C8,C9,C10,C11,C12,C13)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="12">
-        <f>_xll.qlRateHelperQuote(B14)</f>
-        <v>0.3</v>
-      </c>
-      <c r="C15" s="12">
-        <f>_xll.qlRateHelperQuote(C14)</f>
-        <v>0.3</v>
+      <c r="B15" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C15" s="12" t="e">
+        <f ca="1">_xll.qlRateHelperQuote(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="11">
-        <f>_xll.qlRateHelperLatestDate(B14)</f>
-        <v>45755</v>
-      </c>
-      <c r="C16" s="11">
-        <f>_xll.qlRateHelperLatestDate(C14)</f>
-        <v>45754</v>
+      <c r="B16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C16" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestDate(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="11">
-        <f>_xll.qlRateHelperEarliestDate(B14)</f>
-        <v>45665</v>
-      </c>
-      <c r="C17" s="11">
-        <f>_xll.qlRateHelperEarliestDate(C14)</f>
-        <v>45664</v>
+      <c r="B17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C17" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperEarliestDate(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="11">
-        <f>_xll.qlRateHelperMaturityDate(B14)</f>
-        <v>45755</v>
-      </c>
-      <c r="C18" s="11">
-        <f>_xll.qlRateHelperMaturityDate(C14)</f>
-        <v>45754</v>
+      <c r="B18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C18" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperMaturityDate(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(B14)</f>
-        <v>45755</v>
-      </c>
-      <c r="C19" s="11">
-        <f>_xll.qlRateHelperLatestRelevantDate(C14)</f>
-        <v>45754</v>
+      <c r="B19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C19" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperLatestRelevantDate(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="11">
-        <f>_xll.qlRateHelperPillarDate(B14)</f>
-        <v>45755</v>
-      </c>
-      <c r="C20" s="11">
-        <f>_xll.qlRateHelperPillarDate(C14)</f>
-        <v>45754</v>
+      <c r="B20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="11" t="e">
+        <f ca="1">_xll.qlRateHelperPillarDate(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="12">
-        <f>_xll.qlFxSwapRateHelperSpot(B14)</f>
-        <v>0.5</v>
-      </c>
-      <c r="C21" s="12">
-        <f>_xll.qlFxSwapRateHelperSpot(C14)</f>
-        <v>0.5</v>
+      <c r="B21" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperSpot(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C21" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperSpot(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperTenor(B14)</f>
-        <v>3M</v>
-      </c>
-      <c r="C22" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperTenor(C14)</f>
-        <v>3M</v>
+      <c r="B22" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperTenor(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C22" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperTenor(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="B23" s="12">
-        <f>_xll.qlFxSwapRateHelperFixingDays(B14)</f>
-        <v>2</v>
-      </c>
-      <c r="C23" s="12">
-        <f>_xll.qlFxSwapRateHelperFixingDays(C14)</f>
-        <v>1</v>
+      <c r="B23" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperFixingDays(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C23" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperFixingDays(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B24" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperCalendar(B14)</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C24" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperCalendar(C14)</f>
-        <v>TARGET</v>
+      <c r="B24" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperCalendar(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C24" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperCalendar(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B25" s="16">
-        <f>_xll.qlFxSwapRateHelperBusinessDayConvention(B14)</f>
-        <v>0</v>
-      </c>
-      <c r="C25" s="16">
-        <f>_xll.qlFxSwapRateHelperBusinessDayConvention(C14)</f>
-        <v>0</v>
+      <c r="B25" s="16" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperBusinessDayConvention(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C25" s="16" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperBusinessDayConvention(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="12" t="b">
-        <f>_xll.qlFxSwapRateHelperEndOfMonth(B14)</f>
-        <v>1</v>
-      </c>
-      <c r="C26" s="12" t="b">
-        <f>_xll.qlFxSwapRateHelperEndOfMonth(C14)</f>
-        <v>0</v>
+      <c r="B26" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperEndOfMonth(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C26" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperEndOfMonth(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B27" s="12" t="b">
-        <f>_xll.qlFxSwapRateHelperIsFxBaseCurrencyCollateralCurrency(B14)</f>
-        <v>1</v>
-      </c>
-      <c r="C27" s="12" t="b">
-        <f>_xll.qlFxSwapRateHelperIsFxBaseCurrencyCollateralCurrency(C14)</f>
-        <v>0</v>
+      <c r="B27" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperIsFxBaseCurrencyCollateralCurrency(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C27" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperIsFxBaseCurrencyCollateralCurrency(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B28" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperTradingCalendar(B14)</f>
-        <v>Null</v>
-      </c>
-      <c r="C28" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperTradingCalendar(C14)</f>
-        <v>TARGET</v>
+      <c r="B28" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperTradingCalendar(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C28" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperTradingCalendar(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperAdjustmentCalendar(B14)</f>
-        <v>JoinHolidays(Null, TARGET)</v>
-      </c>
-      <c r="C29" s="12" t="str">
-        <f>_xll.qlFxSwapRateHelperAdjustmentCalendar(C14)</f>
-        <v>JoinHolidays(TARGET, TARGET)</v>
+      <c r="B29" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperAdjustmentCalendar(B14)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C29" s="12" t="e">
+        <f ca="1">_xll.qlFxSwapRateHelperAdjustmentCalendar(C14)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>